<commit_message>
ref added in manybooks
</commit_message>
<xml_diff>
--- a/jain/books.xlsx
+++ b/jain/books.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\$MainSitePFin\jainlibrary\jain\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{646648AB-7160-4804-9B64-6D1D906F22C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2780BA96-533A-4D8E-8EA5-1C9E86CCF18B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Books" sheetId="1" r:id="rId1"/>
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="149">
   <si>
     <t>BookID</t>
   </si>
@@ -510,12 +510,6 @@
     <t>Aagams</t>
   </si>
   <si>
-    <t>Gujarati/Buddisagar Suri/Explaination/Jain Christian Samvad - Jain Dharma ane khristi dharma no mukablo/index.html</t>
-  </si>
-  <si>
-    <t>Gujarati/Subodhiben Masalia/QnA/Prashnottar Ratnamala Part 2/index.html</t>
-  </si>
-  <si>
     <t>Prashnottar Ratnamala Part 3</t>
   </si>
   <si>
@@ -523,9 +517,6 @@
   </si>
   <si>
     <t>Chandrakant Lodaya(JJS)</t>
-  </si>
-  <si>
-    <t>Gujarati/Chandrakant Lodaya(JJS)/Tattvartha/Jain Vigyan Part 1 to 6/index.html</t>
   </si>
 </sst>
 </file>
@@ -992,7 +983,7 @@
         <v>143</v>
       </c>
       <c r="G3" t="str">
-        <f t="shared" ref="G3:G40" si="0">E3&amp;"/"&amp;D3&amp;"/"&amp;C3&amp;"/"&amp;B3&amp;"/"&amp;B3&amp;".html"</f>
+        <f t="shared" ref="G3:G42" si="0">E3&amp;"/"&amp;D3&amp;"/"&amp;C3&amp;"/"&amp;B3&amp;"/"&amp;B3&amp;".html"</f>
         <v>Gujarati/Aagams/Aanga Aagam/1- Acharanga Sutra Part 2/1- Acharanga Sutra Part 2.html</v>
       </c>
       <c r="H3" t="s">
@@ -2216,8 +2207,9 @@
       <c r="F38" t="s">
         <v>121</v>
       </c>
-      <c r="G38" s="1" t="s">
-        <v>147</v>
+      <c r="G38" t="str">
+        <f t="shared" si="0"/>
+        <v>Gujarati/Subodhiben Masalia/QnA/Prashnottar Ratnamala Part 2/Prashnottar Ratnamala Part 2.html</v>
       </c>
       <c r="H38" t="s">
         <v>125</v>
@@ -2236,7 +2228,7 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C39" t="s">
         <v>121</v>
@@ -2250,7 +2242,7 @@
       <c r="F39" t="s">
         <v>121</v>
       </c>
-      <c r="G39" s="1" t="str">
+      <c r="G39" t="str">
         <f t="shared" si="0"/>
         <v>Gujarati/Subodhiben Masalia/QnA/Prashnottar Ratnamala Part 3/Prashnottar Ratnamala Part 3.html</v>
       </c>
@@ -2320,8 +2312,9 @@
       <c r="F41" t="s">
         <v>135</v>
       </c>
-      <c r="G41" s="1" t="s">
-        <v>146</v>
+      <c r="G41" t="str">
+        <f t="shared" si="0"/>
+        <v>Gujarati/Buddisagar Suri/Explaination/Jain Christian Samvad - Jain Dharma ane khristi dharma no mukablo/Jain Christian Samvad - Jain Dharma ane khristi dharma no mukablo.html</v>
       </c>
       <c r="H41" t="s">
         <v>136</v>
@@ -2343,10 +2336,10 @@
         <v>138</v>
       </c>
       <c r="C42" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D42" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="E42" t="s">
         <v>10</v>
@@ -2354,8 +2347,9 @@
       <c r="F42" t="s">
         <v>139</v>
       </c>
-      <c r="G42" s="1" t="s">
-        <v>151</v>
+      <c r="G42" t="str">
+        <f t="shared" si="0"/>
+        <v>Gujarati/Chandrakant Lodaya(JJS)/Tattvartha/Jain Vigyan Part 1 to 6/Jain Vigyan Part 1 to 6.html</v>
       </c>
       <c r="H42" t="s">
         <v>140</v>

</xml_diff>